<commit_message>
Update live market close quotes, Excel dashboard, and web terminal
</commit_message>
<xml_diff>
--- a/bloomberg_live_remote_dashboard.xlsx
+++ b/bloomberg_live_remote_dashboard.xlsx
@@ -598,7 +598,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Strategy Playbook &amp; Mathematical Risk Framework | Synced: 2026-10-06 16:23:25</t>
+          <t>Strategy Playbook &amp; Mathematical Risk Framework | Synced: 2026-10-06 17:00:22</t>
         </is>
       </c>
     </row>
@@ -1075,7 +1075,7 @@
         <v>1793977839565.65</v>
       </c>
       <c r="U5" s="17" t="n">
-        <v>30717692</v>
+        <v>30765532</v>
       </c>
       <c r="V5" s="21" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
         <v>5765684000000</v>
       </c>
       <c r="U6" s="17" t="n">
-        <v>100692456</v>
+        <v>100816044</v>
       </c>
       <c r="V6" s="21" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
         <v>2764424305367.88</v>
       </c>
       <c r="U7" s="17" t="n">
-        <v>32765498</v>
+        <v>33977199</v>
       </c>
       <c r="V7" s="21" t="inlineStr">
         <is>
@@ -1324,7 +1324,7 @@
         <v>337782892823.04</v>
       </c>
       <c r="U8" s="17" t="n">
-        <v>4800153</v>
+        <v>5037439</v>
       </c>
       <c r="V8" s="21" t="inlineStr">
         <is>
@@ -1407,7 +1407,7 @@
         <v>321011465897.0699</v>
       </c>
       <c r="U9" s="17" t="n">
-        <v>3426796</v>
+        <v>3516920</v>
       </c>
       <c r="V9" s="21" t="inlineStr">
         <is>
@@ -1490,7 +1490,7 @@
         <v>247030590213.76</v>
       </c>
       <c r="U10" s="17" t="n">
-        <v>4168604</v>
+        <v>4249696</v>
       </c>
       <c r="V10" s="21" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
         <v>271597312723.5</v>
       </c>
       <c r="U11" s="17" t="n">
-        <v>2046129</v>
+        <v>2048447</v>
       </c>
       <c r="V11" s="21" t="inlineStr">
         <is>
@@ -1656,7 +1656,7 @@
         <v>117730978920.36</v>
       </c>
       <c r="U12" s="17" t="n">
-        <v>849370</v>
+        <v>849913</v>
       </c>
       <c r="V12" s="21" t="inlineStr">
         <is>
@@ -1739,7 +1739,7 @@
         <v>4233757895000</v>
       </c>
       <c r="U13" s="17" t="n">
-        <v>18348087</v>
+        <v>18384721</v>
       </c>
       <c r="V13" s="21" t="inlineStr">
         <is>
@@ -1822,7 +1822,7 @@
         <v>850497597035.2</v>
       </c>
       <c r="U14" s="17" t="n">
-        <v>21668064</v>
+        <v>22007285</v>
       </c>
       <c r="V14" s="21" t="inlineStr">
         <is>
@@ -1905,7 +1905,7 @@
         <v>496438404512.4</v>
       </c>
       <c r="U15" s="17" t="n">
-        <v>2286490</v>
+        <v>2286501</v>
       </c>
       <c r="V15" s="21" t="inlineStr">
         <is>
@@ -1988,7 +1988,7 @@
         <v>396901686158.16</v>
       </c>
       <c r="U16" s="17" t="n">
-        <v>1961592</v>
+        <v>1971275</v>
       </c>
       <c r="V16" s="21" t="inlineStr">
         <is>
@@ -2071,7 +2071,7 @@
         <v>1089611389166.85</v>
       </c>
       <c r="U17" s="17" t="n">
-        <v>2123444</v>
+        <v>2130132</v>
       </c>
       <c r="V17" s="21" t="inlineStr">
         <is>
@@ -2154,7 +2154,7 @@
         <v>414727996160</v>
       </c>
       <c r="U18" s="17" t="n">
-        <v>1802700</v>
+        <v>1899700</v>
       </c>
       <c r="V18" s="21" t="inlineStr">
         <is>
@@ -2237,7 +2237,7 @@
         <v>692026707479.2531</v>
       </c>
       <c r="U19" s="17" t="n">
-        <v>3532182</v>
+        <v>3534133</v>
       </c>
       <c r="V19" s="21" t="inlineStr">
         <is>
@@ -2320,7 +2320,7 @@
         <v>880603922679.5999</v>
       </c>
       <c r="U20" s="17" t="n">
-        <v>5835540</v>
+        <v>6286202</v>
       </c>
       <c r="V20" s="21" t="inlineStr">
         <is>
@@ -2403,7 +2403,7 @@
         <v>613993964543.6599</v>
       </c>
       <c r="U21" s="17" t="n">
-        <v>5466086</v>
+        <v>5660662</v>
       </c>
       <c r="V21" s="21" t="inlineStr">
         <is>
@@ -2486,7 +2486,7 @@
         <v>3930341228386.3</v>
       </c>
       <c r="U22" s="17" t="n">
-        <v>20943282</v>
+        <v>21085135</v>
       </c>
       <c r="V22" s="21" t="inlineStr">
         <is>
@@ -2569,7 +2569,7 @@
         <v>410130601056.92</v>
       </c>
       <c r="U23" s="17" t="n">
-        <v>5380136</v>
+        <v>5468327</v>
       </c>
       <c r="V23" s="21" t="inlineStr">
         <is>
@@ -2652,7 +2652,7 @@
         <v>1882301399528</v>
       </c>
       <c r="U24" s="17" t="n">
-        <v>12122803</v>
+        <v>12543646</v>
       </c>
       <c r="V24" s="21" t="inlineStr">
         <is>
@@ -2735,7 +2735,7 @@
         <v>471272508736.65</v>
       </c>
       <c r="U25" s="17" t="n">
-        <v>4411586</v>
+        <v>4500599</v>
       </c>
       <c r="V25" s="21" t="inlineStr">
         <is>
@@ -2818,7 +2818,7 @@
         <v>681680050508.7999</v>
       </c>
       <c r="U26" s="17" t="n">
-        <v>9275314</v>
+        <v>9284710</v>
       </c>
       <c r="V26" s="21" t="inlineStr">
         <is>
@@ -2901,7 +2901,7 @@
         <v>1503513701947.92</v>
       </c>
       <c r="U27" s="17" t="n">
-        <v>27600022</v>
+        <v>27651584</v>
       </c>
       <c r="V27" s="21" t="inlineStr">
         <is>
@@ -2984,7 +2984,7 @@
         <v>4869056273400</v>
       </c>
       <c r="U28" s="17" t="n">
-        <v>29570995</v>
+        <v>30422342</v>
       </c>
       <c r="V28" s="21" t="inlineStr">
         <is>
@@ -3067,7 +3067,7 @@
         <v>1060161941775.64</v>
       </c>
       <c r="U29" s="17" t="n">
-        <v>24153966</v>
+        <v>24185063</v>
       </c>
       <c r="V29" s="21" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add Live vs Offline feed detection, Friend pull launcher, and desktop sync tools
</commit_message>
<xml_diff>
--- a/bloomberg_live_remote_dashboard.xlsx
+++ b/bloomberg_live_remote_dashboard.xlsx
@@ -598,7 +598,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Strategy Playbook &amp; Mathematical Risk Framework | Synced: 2026-10-06 17:00:22</t>
+          <t>Strategy Playbook &amp; Mathematical Risk Framework | Synced: 2026-10-09 14:47:38</t>
         </is>
       </c>
     </row>
@@ -853,7 +853,7 @@
     <col width="29" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
@@ -868,8 +868,8 @@
     <col width="15" customWidth="1" min="17" max="17"/>
     <col width="21" customWidth="1" min="18" max="18"/>
     <col width="21" customWidth="1" min="19" max="19"/>
-    <col width="21" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
     <col width="16" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
@@ -1017,13 +1017,13 @@
         </is>
       </c>
       <c r="D5" s="13" t="n">
-        <v>375.81</v>
+        <v>362.57</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>0.03668864</v>
+        <v>0.006747376</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>0.0583216</v>
+        <v>0.02092133</v>
       </c>
       <c r="G5" s="13" t="n">
         <v>529.7020874023438</v>
@@ -1069,13 +1069,13 @@
         <v>44.24543410014627</v>
       </c>
       <c r="S5" s="19" t="n">
-        <v>45.08017202445418</v>
+        <v>43.49197309083039</v>
       </c>
       <c r="T5" s="20" t="n">
-        <v>1793977839565.65</v>
+        <v>1730774980153.05</v>
       </c>
       <c r="U5" s="17" t="n">
-        <v>30765532</v>
+        <v>12447287</v>
       </c>
       <c r="V5" s="21" t="inlineStr">
         <is>
@@ -1100,16 +1100,16 @@
         </is>
       </c>
       <c r="D6" s="13" t="n">
-        <v>239.24</v>
+        <v>229.785</v>
       </c>
       <c r="E6" s="14" t="n">
-        <v>0.00142319</v>
+        <v>-0.003015446</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>0.05294661</v>
+        <v>-0.01780295</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>323.8887634277344</v>
+        <v>324.6381530761719</v>
       </c>
       <c r="H6" s="14">
         <f>(G6-D6)/D6</f>
@@ -1152,13 +1152,13 @@
         <v>117.210701426553</v>
       </c>
       <c r="S6" s="19" t="n">
-        <v>34.40189614394557</v>
+        <v>33.04229915529706</v>
       </c>
       <c r="T6" s="20" t="n">
-        <v>5765684000000</v>
+        <v>5537818500000</v>
       </c>
       <c r="U6" s="17" t="n">
-        <v>100816044</v>
+        <v>64209802</v>
       </c>
       <c r="V6" s="21" t="inlineStr">
         <is>
@@ -1169,30 +1169,30 @@
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>GE</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>AMAZON.COM INC</t>
+          <t>GENERAL ELECTRIC</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D7" s="13" t="n">
-        <v>256.29</v>
+        <v>307.865</v>
       </c>
       <c r="E7" s="14" t="n">
-        <v>0.01945107</v>
+        <v>0.007345722999999999</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>0.03899947</v>
+        <v>-0.005475514</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>332.6354675292969</v>
+        <v>393</v>
       </c>
       <c r="H7" s="14">
         <f>(G7-D7)/D7</f>
@@ -1219,63 +1219,63 @@
         <v/>
       </c>
       <c r="N7" s="17" t="n">
-        <v>77</v>
+        <v>21</v>
       </c>
       <c r="O7" s="17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P7" s="17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q7" s="14">
         <f>IF((N7+O7+P7)&gt;0, N7/(N7+O7+P7), 0)</f>
         <v/>
       </c>
       <c r="R7" s="18" t="n">
-        <v>30.55833836875067</v>
+        <v>48.79401767505099</v>
       </c>
       <c r="S7" s="19" t="n">
-        <v>35.60544799108563</v>
+        <v>42.63271516035753</v>
       </c>
       <c r="T7" s="20" t="n">
-        <v>2764424305367.88</v>
+        <v>319429183064.745</v>
       </c>
       <c r="U7" s="17" t="n">
-        <v>33977199</v>
+        <v>1844198</v>
       </c>
       <c r="V7" s="21" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>UNITEDHEALTH GROUP INC</t>
+          <t>AMAZON.COM INC</t>
         </is>
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D8" s="13" t="n">
-        <v>376.32</v>
+        <v>261.78</v>
       </c>
       <c r="E8" s="14" t="n">
-        <v>-0.005969676</v>
+        <v>0.03038652</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>0.003680589</v>
+        <v>0.04079198</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>481.1111145019531</v>
+        <v>332.6354675292969</v>
       </c>
       <c r="H8" s="14">
         <f>(G8-D8)/D8</f>
@@ -1302,10 +1302,10 @@
         <v/>
       </c>
       <c r="N8" s="17" t="n">
-        <v>25</v>
+        <v>77</v>
       </c>
       <c r="O8" s="17" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P8" s="17" t="n">
         <v>0</v>
@@ -1315,50 +1315,50 @@
         <v/>
       </c>
       <c r="R8" s="18" t="n">
-        <v>14.62124231898163</v>
+        <v>30.55833836875067</v>
       </c>
       <c r="S8" s="19" t="n">
-        <v>21.13110879776216</v>
+        <v>36.36815256498377</v>
       </c>
       <c r="T8" s="20" t="n">
-        <v>337782892823.04</v>
+        <v>2823641166878.16</v>
       </c>
       <c r="U8" s="17" t="n">
-        <v>5037439</v>
+        <v>24552192</v>
       </c>
       <c r="V8" s="21" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>GE</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>GENERAL ELECTRIC</t>
+          <t>UNITEDHEALTH GROUP INC</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="D9" s="13" t="n">
-        <v>309.39</v>
+        <v>381.71</v>
       </c>
       <c r="E9" s="14" t="n">
-        <v>0.009956258000000001</v>
+        <v>0.0290066</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>-0.02673881</v>
+        <v>0.02637806</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>393</v>
+        <v>480.0740661621094</v>
       </c>
       <c r="H9" s="14">
         <f>(G9-D9)/D9</f>
@@ -1385,45 +1385,45 @@
         <v/>
       </c>
       <c r="N9" s="17" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="O9" s="17" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P9" s="17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q9" s="14">
         <f>IF((N9+O9+P9)&gt;0, N9/(N9+O9+P9), 0)</f>
         <v/>
       </c>
       <c r="R9" s="18" t="n">
-        <v>48.79401767505099</v>
+        <v>14.62124231898163</v>
       </c>
       <c r="S9" s="19" t="n">
-        <v>42.84389841769323</v>
+        <v>21.43376701117273</v>
       </c>
       <c r="T9" s="20" t="n">
-        <v>321011465897.0699</v>
+        <v>342620929048.37</v>
       </c>
       <c r="U9" s="17" t="n">
-        <v>3516920</v>
+        <v>5250799</v>
       </c>
       <c r="V9" s="21" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>RTX</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>RTX CORP</t>
+          <t>CATERPILLAR INC</t>
         </is>
       </c>
       <c r="C10" s="12" t="inlineStr">
@@ -1432,16 +1432,16 @@
         </is>
       </c>
       <c r="D10" s="13" t="n">
-        <v>183.29</v>
+        <v>802.34</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>-0.005642055</v>
+        <v>0.007736944</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>-0.01952498</v>
+        <v>-0.05095692</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>230.5652160644531</v>
+        <v>1007.163208007812</v>
       </c>
       <c r="H10" s="14">
         <f>(G10-D10)/D10</f>
@@ -1468,63 +1468,63 @@
         <v/>
       </c>
       <c r="N10" s="17" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="O10" s="17" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="P10" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q10" s="14">
         <f>IF((N10+O10+P10)&gt;0, N10/(N10+O10+P10), 0)</f>
         <v/>
       </c>
       <c r="R10" s="18" t="n">
-        <v>12.01786060959037</v>
+        <v>56.98969939037208</v>
       </c>
       <c r="S10" s="19" t="n">
-        <v>26.4909171208355</v>
+        <v>34.12093026696047</v>
       </c>
       <c r="T10" s="20" t="n">
-        <v>247030590213.76</v>
+        <v>368815550440.26</v>
       </c>
       <c r="U10" s="17" t="n">
-        <v>4249696</v>
+        <v>1027301</v>
       </c>
       <c r="V10" s="21" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-29</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>LMT</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>GOLDMAN SACHS GROUP INC</t>
+          <t>LOCKHEED MARTIN CORP</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D11" s="13" t="n">
-        <v>897.1799999999999</v>
+        <v>509.29</v>
       </c>
       <c r="E11" s="14" t="n">
-        <v>0.004163589</v>
+        <v>0.002756502</v>
       </c>
       <c r="F11" s="14" t="n">
-        <v>-0.02080241</v>
+        <v>0.007676936</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>1123.772705078125</v>
+        <v>634.0416870117188</v>
       </c>
       <c r="H11" s="14">
         <f>(G11-D11)/D11</f>
@@ -1551,10 +1551,10 @@
         <v/>
       </c>
       <c r="N11" s="17" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O11" s="17" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="P11" s="17" t="n">
         <v>1</v>
@@ -1564,50 +1564,50 @@
         <v/>
       </c>
       <c r="R11" s="18" t="n">
-        <v>18.3355666637702</v>
+        <v>89.16465749539071</v>
       </c>
       <c r="S11" s="19" t="n">
-        <v>13.72168011061556</v>
+        <v>23.50835059235798</v>
       </c>
       <c r="T11" s="20" t="n">
-        <v>271597312723.5</v>
+        <v>117539422595.37</v>
       </c>
       <c r="U11" s="17" t="n">
-        <v>2048447</v>
+        <v>519730</v>
       </c>
       <c r="V11" s="21" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>LMT</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>LOCKHEED MARTIN CORP</t>
+          <t>GOLDMAN SACHS GROUP INC</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D12" s="13" t="n">
-        <v>510.12</v>
+        <v>897.14</v>
       </c>
       <c r="E12" s="14" t="n">
-        <v>0.006888656</v>
+        <v>0.01648557</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>-0.004080358</v>
+        <v>-0.006005141</v>
       </c>
       <c r="G12" s="13" t="n">
-        <v>638.8261108398438</v>
+        <v>1116</v>
       </c>
       <c r="H12" s="14">
         <f>(G12-D12)/D12</f>
@@ -1634,10 +1634,10 @@
         <v/>
       </c>
       <c r="N12" s="17" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="O12" s="17" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="P12" s="17" t="n">
         <v>1</v>
@@ -1647,50 +1647,50 @@
         <v/>
       </c>
       <c r="R12" s="18" t="n">
-        <v>89.16465749539071</v>
+        <v>18.3355666637702</v>
       </c>
       <c r="S12" s="19" t="n">
-        <v>23.54666199647038</v>
+        <v>13.72106867733892</v>
       </c>
       <c r="T12" s="20" t="n">
-        <v>117730978920.36</v>
+        <v>271585203790.5</v>
       </c>
       <c r="U12" s="17" t="n">
-        <v>849913</v>
+        <v>1280873</v>
       </c>
       <c r="V12" s="21" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>RTX</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>ALPHABET INC-CL A</t>
+          <t>RTX CORP</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D13" s="13" t="n">
-        <v>347.68</v>
+        <v>185.75</v>
       </c>
       <c r="E13" s="14" t="n">
-        <v>0.003492366</v>
+        <v>0.007758247</v>
       </c>
       <c r="F13" s="14" t="n">
-        <v>0.0198287</v>
+        <v>0.005793806</v>
       </c>
       <c r="G13" s="13" t="n">
-        <v>429.2468566894531</v>
+        <v>229.625</v>
       </c>
       <c r="H13" s="14">
         <f>(G13-D13)/D13</f>
@@ -1717,63 +1717,63 @@
         <v/>
       </c>
       <c r="N13" s="17" t="n">
-        <v>64</v>
+        <v>20</v>
       </c>
       <c r="O13" s="17" t="n">
         <v>7</v>
       </c>
       <c r="P13" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q13" s="14">
         <f>IF((N13+O13+P13)&gt;0, N13/(N13+O13+P13), 0)</f>
         <v/>
       </c>
       <c r="R13" s="18" t="n">
-        <v>49.54854659098636</v>
+        <v>12.01786060959037</v>
       </c>
       <c r="S13" s="19" t="n">
-        <v>33.61601864774237</v>
+        <v>26.84646208434053</v>
       </c>
       <c r="T13" s="20" t="n">
-        <v>4233757895000</v>
+        <v>250346075248</v>
       </c>
       <c r="U13" s="17" t="n">
-        <v>18384721</v>
+        <v>2282384</v>
       </c>
       <c r="V13" s="21" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>WALMART INC</t>
+          <t>ALPHABET INC-CL A</t>
         </is>
       </c>
       <c r="C14" s="12" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="D14" s="13" t="n">
-        <v>107.2</v>
+        <v>351.23</v>
       </c>
       <c r="E14" s="14" t="n">
-        <v>0.0202722</v>
+        <v>0.008441241</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>0.003745318</v>
+        <v>0.02250364</v>
       </c>
       <c r="G14" s="13" t="n">
-        <v>128.2888946533203</v>
+        <v>429.2468566894531</v>
       </c>
       <c r="H14" s="14">
         <f>(G14-D14)/D14</f>
@@ -1800,63 +1800,63 @@
         <v/>
       </c>
       <c r="N14" s="17" t="n">
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="O14" s="17" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="P14" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q14" s="14">
         <f>IF((N14+O14+P14)&gt;0, N14/(N14+O14+P14), 0)</f>
         <v/>
       </c>
       <c r="R14" s="18" t="n">
-        <v>23.4417142735787</v>
+        <v>49.54854659098636</v>
       </c>
       <c r="S14" s="19" t="n">
-        <v>37.90012008124562</v>
+        <v>33.95925807549528</v>
       </c>
       <c r="T14" s="20" t="n">
-        <v>850497597035.2</v>
+        <v>4274231867500</v>
       </c>
       <c r="U14" s="17" t="n">
-        <v>22007285</v>
+        <v>11846311</v>
       </c>
       <c r="V14" s="21" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>MASTERCARD INC - A</t>
+          <t>WALMART INC</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D15" s="13" t="n">
-        <v>566.58</v>
+        <v>111.145</v>
       </c>
       <c r="E15" s="14" t="n">
-        <v>0.003524682</v>
+        <v>0.005291245</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>0.005323113000000001</v>
+        <v>0.06603683</v>
       </c>
       <c r="G15" s="13" t="n">
-        <v>670.5609741210938</v>
+        <v>128.8444519042969</v>
       </c>
       <c r="H15" s="14">
         <f>(G15-D15)/D15</f>
@@ -1886,60 +1886,60 @@
         <v>46</v>
       </c>
       <c r="O15" s="17" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P15" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q15" s="14">
         <f>IF((N15+O15+P15)&gt;0, N15/(N15+O15+P15), 0)</f>
         <v/>
       </c>
       <c r="R15" s="18" t="n">
-        <v>241.4884135472371</v>
+        <v>23.4417142735787</v>
       </c>
       <c r="S15" s="19" t="n">
-        <v>29.88450109002861</v>
+        <v>39.29485857388293</v>
       </c>
       <c r="T15" s="20" t="n">
-        <v>496438404512.4</v>
+        <v>881796225955.9449</v>
       </c>
       <c r="U15" s="17" t="n">
-        <v>2286501</v>
+        <v>7916610</v>
       </c>
       <c r="V15" s="21" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-11-19</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t>CATERPILLAR INC</t>
+          <t>ELI LILLY &amp; CO</t>
         </is>
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="D16" s="13" t="n">
-        <v>863.4400000000001</v>
+        <v>1175.95</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>0.01803947</v>
+        <v>0.005429207</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>0.04451757</v>
+        <v>0.02896268</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>1007.163208007812</v>
+        <v>1347.217529296875</v>
       </c>
       <c r="H16" s="14">
         <f>(G16-D16)/D16</f>
@@ -1966,29 +1966,29 @@
         <v/>
       </c>
       <c r="N16" s="17" t="n">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="O16" s="17" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="P16" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q16" s="14">
         <f>IF((N16+O16+P16)&gt;0, N16/(N16+O16+P16), 0)</f>
         <v/>
       </c>
       <c r="R16" s="18" t="n">
-        <v>56.98969939037208</v>
+        <v>102.4296334361739</v>
       </c>
       <c r="S16" s="19" t="n">
-        <v>36.71931491249718</v>
+        <v>33.02816049054621</v>
       </c>
       <c r="T16" s="20" t="n">
-        <v>396901686158.16</v>
+        <v>1106988840586.75</v>
       </c>
       <c r="U16" s="17" t="n">
-        <v>1971275</v>
+        <v>924530</v>
       </c>
       <c r="V16" s="21" t="inlineStr">
         <is>
@@ -1999,30 +1999,30 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>LLY</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>ELI LILLY &amp; CO</t>
+          <t>MASTERCARD INC - A</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D17" s="13" t="n">
-        <v>1157.49</v>
+        <v>588.925</v>
       </c>
       <c r="E17" s="14" t="n">
-        <v>0.01257086</v>
+        <v>0.0261984</v>
       </c>
       <c r="F17" s="14" t="n">
-        <v>-0.02291011</v>
+        <v>0.06639083</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>1346.066040039062</v>
+        <v>670.6666870117188</v>
       </c>
       <c r="H17" s="14">
         <f>(G17-D17)/D17</f>
@@ -2049,29 +2049,29 @@
         <v/>
       </c>
       <c r="N17" s="17" t="n">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="O17" s="17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P17" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="14">
         <f>IF((N17+O17+P17)&gt;0, N17/(N17+O17+P17), 0)</f>
         <v/>
       </c>
       <c r="R17" s="18" t="n">
-        <v>102.4296334361739</v>
+        <v>241.4884135472371</v>
       </c>
       <c r="S17" s="19" t="n">
-        <v>32.50968727501066</v>
+        <v>31.06309595958312</v>
       </c>
       <c r="T17" s="20" t="n">
-        <v>1089611389166.85</v>
+        <v>516017133286.5</v>
       </c>
       <c r="U17" s="17" t="n">
-        <v>2130132</v>
+        <v>1543688</v>
       </c>
       <c r="V17" s="21" t="inlineStr">
         <is>
@@ -2096,16 +2096,16 @@
         </is>
       </c>
       <c r="D18" s="13" t="n">
-        <v>935.6799999999999</v>
+        <v>946.9</v>
       </c>
       <c r="E18" s="14" t="n">
-        <v>0.01316701</v>
+        <v>-0.00107604</v>
       </c>
       <c r="F18" s="14" t="n">
-        <v>0.01199451</v>
+        <v>0.02851246</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>1074.228515625</v>
+        <v>1077.085693359375</v>
       </c>
       <c r="H18" s="14">
         <f>(G18-D18)/D18</f>
@@ -2148,13 +2148,13 @@
         <v>28.4021118413964</v>
       </c>
       <c r="S18" s="19" t="n">
-        <v>45.07345741745105</v>
+        <v>45.61394735710621</v>
       </c>
       <c r="T18" s="20" t="n">
-        <v>414727996160</v>
+        <v>419599180568.1</v>
       </c>
       <c r="U18" s="17" t="n">
-        <v>1899700</v>
+        <v>924736</v>
       </c>
       <c r="V18" s="21" t="inlineStr">
         <is>
@@ -2165,12 +2165,12 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>VISA INC-CLASS A SHARES</t>
+          <t>JPMORGAN CHASE &amp; CO</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
@@ -2179,16 +2179,16 @@
         </is>
       </c>
       <c r="D19" s="13" t="n">
-        <v>370.64</v>
+        <v>333.34</v>
       </c>
       <c r="E19" s="14" t="n">
-        <v>0.002515485</v>
+        <v>0.005793253000000001</v>
       </c>
       <c r="F19" s="14" t="n">
-        <v>0.01300973</v>
+        <v>0.00288826</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>424.3902587890625</v>
+        <v>371.4003601074219</v>
       </c>
       <c r="H19" s="14">
         <f>(G19-D19)/D19</f>
@@ -2215,63 +2215,63 @@
         <v/>
       </c>
       <c r="N19" s="17" t="n">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="O19" s="17" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="P19" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q19" s="14">
         <f>IF((N19+O19+P19)&gt;0, N19/(N19+O19+P19), 0)</f>
         <v/>
       </c>
       <c r="R19" s="18" t="n">
-        <v>62.35974440012697</v>
+        <v>18.4323841277336</v>
       </c>
       <c r="S19" s="19" t="n">
-        <v>31.12743601096157</v>
+        <v>14.17862491402675</v>
       </c>
       <c r="T19" s="20" t="n">
-        <v>692026707479.2531</v>
+        <v>886079786241.2998</v>
       </c>
       <c r="U19" s="17" t="n">
-        <v>3534133</v>
+        <v>3168300</v>
       </c>
       <c r="V19" s="21" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B20" s="12" t="inlineStr">
         <is>
-          <t>JPMORGAN CHASE &amp; CO</t>
+          <t>META PLATFORMS INC-CLASS A</t>
         </is>
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="D20" s="13" t="n">
-        <v>331.28</v>
+        <v>719.36</v>
       </c>
       <c r="E20" s="14" t="n">
-        <v>0.001662988</v>
+        <v>-0.002122377</v>
       </c>
       <c r="F20" s="14" t="n">
-        <v>-0.01104544</v>
+        <v>-0.01197671</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>371.915771484375</v>
+        <v>795.2846069335938</v>
       </c>
       <c r="H20" s="14">
         <f>(G20-D20)/D20</f>
@@ -2298,10 +2298,10 @@
         <v/>
       </c>
       <c r="N20" s="17" t="n">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="O20" s="17" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="P20" s="17" t="n">
         <v>1</v>
@@ -2311,50 +2311,50 @@
         <v/>
       </c>
       <c r="R20" s="18" t="n">
-        <v>18.4323841277336</v>
+        <v>29.84849580640424</v>
       </c>
       <c r="S20" s="19" t="n">
-        <v>14.0910028673837</v>
+        <v>21.29844122656482</v>
       </c>
       <c r="T20" s="20" t="n">
-        <v>880603922679.5999</v>
+        <v>1832574078016</v>
       </c>
       <c r="U20" s="17" t="n">
-        <v>6286202</v>
+        <v>9992704</v>
       </c>
       <c r="V20" s="21" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-29</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>JNJ</t>
+          <t>V</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>JOHNSON &amp; JOHNSON</t>
+          <t>VISA INC-CLASS A SHARES</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D21" s="13" t="n">
-        <v>254.78</v>
+        <v>385.245</v>
       </c>
       <c r="E21" s="14" t="n">
-        <v>0.007314277</v>
+        <v>0.02704612</v>
       </c>
       <c r="F21" s="14" t="n">
-        <v>-0.04780058</v>
+        <v>0.06816669</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>284.0400085449219</v>
+        <v>424.2857055664063</v>
       </c>
       <c r="H21" s="14">
         <f>(G21-D21)/D21</f>
@@ -2381,10 +2381,10 @@
         <v/>
       </c>
       <c r="N21" s="17" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="O21" s="17" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P21" s="17" t="n">
         <v>0</v>
@@ -2394,50 +2394,50 @@
         <v/>
       </c>
       <c r="R21" s="18" t="n">
-        <v>25.74215021658794</v>
+        <v>62.35974440012697</v>
       </c>
       <c r="S21" s="19" t="n">
-        <v>27.48902847887283</v>
+        <v>32.354005126586</v>
       </c>
       <c r="T21" s="20" t="n">
-        <v>613993964543.6599</v>
+        <v>719295890683.2638</v>
       </c>
       <c r="U21" s="17" t="n">
-        <v>5660662</v>
+        <v>3837920</v>
       </c>
       <c r="V21" s="21" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>JNJ</t>
         </is>
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>MICROSOFT CORP</t>
+          <t>JOHNSON &amp; JOHNSON</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="D22" s="13" t="n">
-        <v>529.3</v>
+        <v>260.28</v>
       </c>
       <c r="E22" s="14" t="n">
-        <v>0.007844929</v>
+        <v>0.01481597</v>
       </c>
       <c r="F22" s="14" t="n">
-        <v>0.03996385</v>
+        <v>0.01659962</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>580.3292846679688</v>
+        <v>284.2000122070312</v>
       </c>
       <c r="H22" s="14">
         <f>(G22-D22)/D22</f>
@@ -2464,10 +2464,10 @@
         <v/>
       </c>
       <c r="N22" s="17" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="O22" s="17" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="P22" s="17" t="n">
         <v>0</v>
@@ -2477,50 +2477,50 @@
         <v/>
       </c>
       <c r="R22" s="18" t="n">
-        <v>34.03862745048138</v>
+        <v>25.74215021658794</v>
       </c>
       <c r="S22" s="19" t="n">
-        <v>31.89910239509463</v>
+        <v>28.08244105975901</v>
       </c>
       <c r="T22" s="20" t="n">
-        <v>3930341228386.3</v>
+        <v>627248406827.1599</v>
       </c>
       <c r="U22" s="17" t="n">
-        <v>21085135</v>
+        <v>3305448</v>
       </c>
       <c r="V22" s="21" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>CHEVRON CORP</t>
+          <t>MICROSOFT CORP</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D23" s="13" t="n">
-        <v>207.58</v>
+        <v>535.4109999999999</v>
       </c>
       <c r="E23" s="14" t="n">
-        <v>0.005376084</v>
+        <v>0.02449436</v>
       </c>
       <c r="F23" s="14" t="n">
-        <v>0.01565711</v>
+        <v>0.03455065</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>224.0740814208984</v>
+        <v>582.3107299804688</v>
       </c>
       <c r="H23" s="14">
         <f>(G23-D23)/D23</f>
@@ -2547,63 +2547,63 @@
         <v/>
       </c>
       <c r="N23" s="17" t="n">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="O23" s="17" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="P23" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q23" s="14">
         <f>IF((N23+O23+P23)&gt;0, N23/(N23+O23+P23), 0)</f>
         <v/>
       </c>
       <c r="R23" s="18" t="n">
-        <v>12.24561403508772</v>
+        <v>34.03862745048138</v>
       </c>
       <c r="S23" s="19" t="n">
-        <v>20.25740526150474</v>
+        <v>32.2673928755247</v>
       </c>
       <c r="T23" s="20" t="n">
-        <v>410130601056.92</v>
+        <v>3975718736881.8</v>
       </c>
       <c r="U23" s="17" t="n">
-        <v>5468327</v>
+        <v>12457020</v>
       </c>
       <c r="V23" s="21" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>META PLATFORMS INC-CLASS A</t>
+          <t>ADVANCED MICRO DEVICES</t>
         </is>
       </c>
       <c r="C24" s="12" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D24" s="13" t="n">
-        <v>738.88</v>
+        <v>609.7431</v>
       </c>
       <c r="E24" s="14" t="n">
-        <v>-0.004070629</v>
+        <v>-0.01762084</v>
       </c>
       <c r="F24" s="14" t="n">
-        <v>0.0001218208</v>
+        <v>-0.03812355</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>794.490966796875</v>
+        <v>648.9697875976562</v>
       </c>
       <c r="H24" s="14">
         <f>(G24-D24)/D24</f>
@@ -2630,63 +2630,63 @@
         <v/>
       </c>
       <c r="N24" s="17" t="n">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="O24" s="17" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="P24" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q24" s="14">
         <f>IF((N24+O24+P24)&gt;0, N24/(N24+O24+P24), 0)</f>
         <v/>
       </c>
       <c r="R24" s="18" t="n">
-        <v>29.84849580640424</v>
+        <v>10.14114698673644</v>
       </c>
       <c r="S24" s="19" t="n">
-        <v>21.87637994597322</v>
+        <v>169.2992508898463</v>
       </c>
       <c r="T24" s="20" t="n">
-        <v>1882301399528</v>
+        <v>995390392781.7102</v>
       </c>
       <c r="U24" s="17" t="n">
-        <v>12543646</v>
+        <v>10939958</v>
       </c>
       <c r="V24" s="21" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-11-03</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>ABBV</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>ABBVIE INC</t>
+          <t>CHEVRON CORP</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D25" s="13" t="n">
-        <v>266.69</v>
+        <v>211.69</v>
       </c>
       <c r="E25" s="14" t="n">
-        <v>0.003499398</v>
+        <v>0.0006617821</v>
       </c>
       <c r="F25" s="14" t="n">
-        <v>0.01291352</v>
+        <v>0.02419082</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>281.4482727050781</v>
+        <v>225.2142791748047</v>
       </c>
       <c r="H25" s="14">
         <f>(G25-D25)/D25</f>
@@ -2713,29 +2713,29 @@
         <v/>
       </c>
       <c r="N25" s="17" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="O25" s="17" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P25" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q25" s="14">
         <f>IF((N25+O25+P25)&gt;0, N25/(N25+O25+P25), 0)</f>
         <v/>
       </c>
       <c r="R25" s="18" t="n">
-        <v>0</v>
+        <v>12.24561403508772</v>
       </c>
       <c r="S25" s="19" t="n">
-        <v>26.27048745760376</v>
+        <v>20.6584937442801</v>
       </c>
       <c r="T25" s="20" t="n">
-        <v>471272508736.65</v>
+        <v>418251020993.06</v>
       </c>
       <c r="U25" s="17" t="n">
-        <v>4500599</v>
+        <v>3943646</v>
       </c>
       <c r="V25" s="21" t="inlineStr">
         <is>
@@ -2746,30 +2746,30 @@
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>XOM</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>EXXONMOBIL HOLDINGS CORP</t>
+          <t>TESLA INC</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D26" s="13" t="n">
-        <v>164.48</v>
+        <v>383.97</v>
       </c>
       <c r="E26" s="14" t="n">
-        <v>0.002926829</v>
+        <v>0.02392</v>
       </c>
       <c r="F26" s="14" t="n">
-        <v>0.01939882</v>
+        <v>0.03610459</v>
       </c>
       <c r="G26" s="13" t="n">
-        <v>172.4400024414062</v>
+        <v>397.1675109863281</v>
       </c>
       <c r="H26" s="14">
         <f>(G26-D26)/D26</f>
@@ -2796,63 +2796,63 @@
         <v/>
       </c>
       <c r="N26" s="17" t="n">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="O26" s="17" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="P26" s="17" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="Q26" s="14">
         <f>IF((N26+O26+P26)&gt;0, N26/(N26+O26+P26), 0)</f>
         <v/>
       </c>
       <c r="R26" s="18" t="n">
-        <v>12.5512239138806</v>
+        <v>4.636600638354896</v>
       </c>
       <c r="S26" s="19" t="n">
-        <v>19.84385459737762</v>
+        <v>384.1175023416023</v>
       </c>
       <c r="T26" s="20" t="n">
-        <v>681680050508.7999</v>
+        <v>1516507712874.18</v>
       </c>
       <c r="U26" s="17" t="n">
-        <v>9284710</v>
+        <v>33777365</v>
       </c>
       <c r="V26" s="21" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>ABBV</t>
         </is>
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>TESLA INC</t>
+          <t>ABBVIE INC</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="D27" s="13" t="n">
-        <v>380.68</v>
+        <v>276.12</v>
       </c>
       <c r="E27" s="14" t="n">
-        <v>0.005148787</v>
+        <v>0.01358197</v>
       </c>
       <c r="F27" s="14" t="n">
-        <v>0.07890261999999999</v>
+        <v>0.05060498</v>
       </c>
       <c r="G27" s="13" t="n">
-        <v>393.6597595214844</v>
+        <v>283.1724243164062</v>
       </c>
       <c r="H27" s="14">
         <f>(G27-D27)/D27</f>
@@ -2879,63 +2879,63 @@
         <v/>
       </c>
       <c r="N27" s="17" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="O27" s="17" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="P27" s="17" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="Q27" s="14">
         <f>IF((N27+O27+P27)&gt;0, N27/(N27+O27+P27), 0)</f>
         <v/>
       </c>
       <c r="R27" s="18" t="n">
-        <v>4.636600638354896</v>
+        <v>0</v>
       </c>
       <c r="S27" s="19" t="n">
-        <v>380.8262299480813</v>
+        <v>27.19939556081934</v>
       </c>
       <c r="T27" s="20" t="n">
-        <v>1503513701947.92</v>
+        <v>487936424734.2</v>
       </c>
       <c r="U27" s="17" t="n">
-        <v>27651584</v>
+        <v>2057977</v>
       </c>
       <c r="V27" s="21" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>XOM</t>
         </is>
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>APPLE INC</t>
+          <t>EXXONMOBIL HOLDINGS CORP</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D28" s="13" t="n">
-        <v>333.63</v>
+        <v>168.77</v>
       </c>
       <c r="E28" s="14" t="n">
-        <v>0.002222957</v>
+        <v>0.001602374</v>
       </c>
       <c r="F28" s="14" t="n">
-        <v>0.01284153</v>
+        <v>0.02902262</v>
       </c>
       <c r="G28" s="13" t="n">
-        <v>333.6066589355469</v>
+        <v>172.6399993896484</v>
       </c>
       <c r="H28" s="14">
         <f>(G28-D28)/D28</f>
@@ -2962,45 +2962,45 @@
         <v/>
       </c>
       <c r="N28" s="17" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="O28" s="17" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="P28" s="17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q28" s="14">
         <f>IF((N28+O28+P28)&gt;0, N28/(N28+O28+P28), 0)</f>
         <v/>
       </c>
       <c r="R28" s="18" t="n">
-        <v>148.7510816267667</v>
+        <v>12.5512239138806</v>
       </c>
       <c r="S28" s="19" t="n">
-        <v>38.260321660873</v>
+        <v>20.36142699522687</v>
       </c>
       <c r="T28" s="20" t="n">
-        <v>4869056273400</v>
+        <v>699459764861.2001</v>
       </c>
       <c r="U28" s="17" t="n">
-        <v>30422342</v>
+        <v>5493118</v>
       </c>
       <c r="V28" s="21" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-11-27</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>ADVANCED MICRO DEVICES</t>
+          <t>APPLE INC</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
@@ -3009,16 +3009,16 @@
         </is>
       </c>
       <c r="D29" s="13" t="n">
-        <v>649.42</v>
+        <v>337.0814</v>
       </c>
       <c r="E29" s="14" t="n">
-        <v>0.02796992</v>
+        <v>-0.009807297</v>
       </c>
       <c r="F29" s="14" t="n">
-        <v>0.06888095</v>
+        <v>0.01016333</v>
       </c>
       <c r="G29" s="13" t="n">
-        <v>648.9697875976562</v>
+        <v>333.6066589355469</v>
       </c>
       <c r="H29" s="14">
         <f>(G29-D29)/D29</f>
@@ -3045,33 +3045,33 @@
         <v/>
       </c>
       <c r="N29" s="17" t="n">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="O29" s="17" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="P29" s="17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q29" s="14">
         <f>IF((N29+O29+P29)&gt;0, N29/(N29+O29+P29), 0)</f>
         <v/>
       </c>
       <c r="R29" s="18" t="n">
-        <v>10.14114698673644</v>
+        <v>148.7510816267667</v>
       </c>
       <c r="S29" s="19" t="n">
-        <v>180.3158019725165</v>
+        <v>38.65612275009856</v>
       </c>
       <c r="T29" s="20" t="n">
-        <v>1060161941775.64</v>
+        <v>4919426626251.999</v>
       </c>
       <c r="U29" s="17" t="n">
-        <v>24185063</v>
+        <v>29097798</v>
       </c>
       <c r="V29" s="21" t="inlineStr">
         <is>
-          <t>2026-11-04</t>
+          <t>2026-11-02</t>
         </is>
       </c>
     </row>
@@ -3607,7 +3607,7 @@
         </is>
       </c>
       <c r="D5" s="13" t="n">
-        <v>331.28</v>
+        <v>333.34</v>
       </c>
       <c r="E5" s="21" t="inlineStr">
         <is>
@@ -3615,14 +3615,14 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>371.915771484375</v>
+        <v>371.4003601074219</v>
       </c>
       <c r="G5" s="14">
         <f>(F5-D5)/D5</f>
         <v/>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.5151515151515151</v>
+        <v>0.5</v>
       </c>
       <c r="I5" s="16">
         <f>IF(G5&gt;=0.25, "HIGH CONVICTION CATALYST", IF(G5&gt;=0.10, "MONITORING CATALYST", "SECONDARY"))</f>
@@ -3632,12 +3632,12 @@
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>JNJ</t>
         </is>
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>UNITEDHEALTH GROUP INC</t>
+          <t>JOHNSON &amp; JOHNSON</t>
         </is>
       </c>
       <c r="C6" s="12" t="inlineStr">
@@ -3646,7 +3646,7 @@
         </is>
       </c>
       <c r="D6" s="13" t="n">
-        <v>376.32</v>
+        <v>260.28</v>
       </c>
       <c r="E6" s="21" t="inlineStr">
         <is>
@@ -3654,14 +3654,14 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>481.1111145019531</v>
+        <v>284.2000122070312</v>
       </c>
       <c r="G6" s="14">
         <f>(F6-D6)/D6</f>
         <v/>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.7407407407407407</v>
       </c>
       <c r="I6" s="16">
         <f>IF(G6&gt;=0.25, "HIGH CONVICTION CATALYST", IF(G6&gt;=0.10, "MONITORING CATALYST", "SECONDARY"))</f>
@@ -3685,7 +3685,7 @@
         </is>
       </c>
       <c r="D7" s="13" t="n">
-        <v>897.1799999999999</v>
+        <v>897.14</v>
       </c>
       <c r="E7" s="21" t="inlineStr">
         <is>
@@ -3693,14 +3693,14 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>1123.772705078125</v>
+        <v>1116</v>
       </c>
       <c r="G7" s="14">
         <f>(F7-D7)/D7</f>
         <v/>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.3928571428571428</v>
+        <v>0.4137931034482759</v>
       </c>
       <c r="I7" s="16">
         <f>IF(G7&gt;=0.25, "HIGH CONVICTION CATALYST", IF(G7&gt;=0.10, "MONITORING CATALYST", "SECONDARY"))</f>
@@ -3710,12 +3710,12 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>JNJ</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>JOHNSON &amp; JOHNSON</t>
+          <t>UNITEDHEALTH GROUP INC</t>
         </is>
       </c>
       <c r="C8" s="12" t="inlineStr">
@@ -3724,7 +3724,7 @@
         </is>
       </c>
       <c r="D8" s="13" t="n">
-        <v>254.78</v>
+        <v>381.71</v>
       </c>
       <c r="E8" s="21" t="inlineStr">
         <is>
@@ -3732,14 +3732,14 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>284.0400085449219</v>
+        <v>480.0740661621094</v>
       </c>
       <c r="G8" s="14">
         <f>(F8-D8)/D8</f>
         <v/>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7407407407407407</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="I8" s="16">
         <f>IF(G8&gt;=0.25, "HIGH CONVICTION CATALYST", IF(G8&gt;=0.10, "MONITORING CATALYST", "SECONDARY"))</f>
@@ -3763,7 +3763,7 @@
         </is>
       </c>
       <c r="D9" s="13" t="n">
-        <v>183.29</v>
+        <v>185.75</v>
       </c>
       <c r="E9" s="21" t="inlineStr">
         <is>
@@ -3771,14 +3771,14 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>230.5652160644531</v>
+        <v>229.625</v>
       </c>
       <c r="G9" s="14">
         <f>(F9-D9)/D9</f>
         <v/>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7037037037037037</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="I9" s="16">
         <f>IF(G9&gt;=0.25, "HIGH CONVICTION CATALYST", IF(G9&gt;=0.10, "MONITORING CATALYST", "SECONDARY"))</f>
@@ -3802,7 +3802,7 @@
         </is>
       </c>
       <c r="D10" s="13" t="n">
-        <v>309.39</v>
+        <v>307.865</v>
       </c>
       <c r="E10" s="21" t="inlineStr">
         <is>
@@ -3841,7 +3841,7 @@
         </is>
       </c>
       <c r="D11" s="13" t="n">
-        <v>380.68</v>
+        <v>383.97</v>
       </c>
       <c r="E11" s="21" t="inlineStr">
         <is>
@@ -3849,7 +3849,7 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>393.6597595214844</v>
+        <v>397.1675109863281</v>
       </c>
       <c r="G11" s="14">
         <f>(F11-D11)/D11</f>
@@ -3880,7 +3880,7 @@
         </is>
       </c>
       <c r="D12" s="13" t="n">
-        <v>510.12</v>
+        <v>509.29</v>
       </c>
       <c r="E12" s="21" t="inlineStr">
         <is>
@@ -3888,14 +3888,14 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>638.8261108398438</v>
+        <v>634.0416870117188</v>
       </c>
       <c r="G12" s="14">
         <f>(F12-D12)/D12</f>
         <v/>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.4814814814814815</v>
+        <v>0.4642857142857143</v>
       </c>
       <c r="I12" s="16">
         <f>IF(G12&gt;=0.25, "HIGH CONVICTION CATALYST", IF(G12&gt;=0.10, "MONITORING CATALYST", "SECONDARY"))</f>
@@ -3919,15 +3919,15 @@
         </is>
       </c>
       <c r="D13" s="13" t="n">
-        <v>370.64</v>
+        <v>385.245</v>
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>424.3902587890625</v>
+        <v>424.2857055664063</v>
       </c>
       <c r="G13" s="14">
         <f>(F13-D13)/D13</f>
@@ -3958,7 +3958,7 @@
         </is>
       </c>
       <c r="D14" s="13" t="n">
-        <v>347.68</v>
+        <v>351.23</v>
       </c>
       <c r="E14" s="21" t="inlineStr">
         <is>
@@ -3983,36 +3983,36 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>CATERPILLAR INC</t>
+          <t>MICROSOFT CORP</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D15" s="13" t="n">
-        <v>863.4400000000001</v>
+        <v>535.4109999999999</v>
       </c>
       <c r="E15" s="21" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>1007.163208007812</v>
+        <v>582.3107299804688</v>
       </c>
       <c r="G15" s="14">
         <f>(F15-D15)/D15</f>
         <v/>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.6071428571428571</v>
+        <v>0.9722222222222222</v>
       </c>
       <c r="I15" s="16">
         <f>IF(G15&gt;=0.25, "HIGH CONVICTION CATALYST", IF(G15&gt;=0.10, "MONITORING CATALYST", "SECONDARY"))</f>
@@ -4022,21 +4022,21 @@
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t>MICROSOFT CORP</t>
+          <t>META PLATFORMS INC-CLASS A</t>
         </is>
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="D16" s="13" t="n">
-        <v>529.3</v>
+        <v>719.36</v>
       </c>
       <c r="E16" s="21" t="inlineStr">
         <is>
@@ -4044,14 +4044,14 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>580.3292846679688</v>
+        <v>795.2846069335938</v>
       </c>
       <c r="G16" s="14">
         <f>(F16-D16)/D16</f>
         <v/>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.9722222222222222</v>
+        <v>0.9113924050632911</v>
       </c>
       <c r="I16" s="16">
         <f>IF(G16&gt;=0.25, "HIGH CONVICTION CATALYST", IF(G16&gt;=0.10, "MONITORING CATALYST", "SECONDARY"))</f>
@@ -4061,21 +4061,21 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>META PLATFORMS INC-CLASS A</t>
+          <t>ELI LILLY &amp; CO</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="D17" s="13" t="n">
-        <v>738.88</v>
+        <v>1175.95</v>
       </c>
       <c r="E17" s="21" t="inlineStr">
         <is>
@@ -4083,14 +4083,14 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>794.490966796875</v>
+        <v>1347.217529296875</v>
       </c>
       <c r="G17" s="14">
         <f>(F17-D17)/D17</f>
         <v/>
       </c>
       <c r="H17" s="14" t="n">
-        <v>0.9113924050632911</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="I17" s="16">
         <f>IF(G17&gt;=0.25, "HIGH CONVICTION CATALYST", IF(G17&gt;=0.10, "MONITORING CATALYST", "SECONDARY"))</f>
@@ -4100,21 +4100,21 @@
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>LLY</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>ELI LILLY &amp; CO</t>
+          <t>MASTERCARD INC - A</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D18" s="13" t="n">
-        <v>1157.49</v>
+        <v>588.925</v>
       </c>
       <c r="E18" s="21" t="inlineStr">
         <is>
@@ -4122,14 +4122,14 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>1346.066040039062</v>
+        <v>670.6666870117188</v>
       </c>
       <c r="G18" s="14">
         <f>(F18-D18)/D18</f>
         <v/>
       </c>
       <c r="H18" s="14" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.9387755102040817</v>
       </c>
       <c r="I18" s="16">
         <f>IF(G18&gt;=0.25, "HIGH CONVICTION CATALYST", IF(G18&gt;=0.10, "MONITORING CATALYST", "SECONDARY"))</f>
@@ -4139,36 +4139,36 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>MASTERCARD INC - A</t>
+          <t>CATERPILLAR INC</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D19" s="13" t="n">
-        <v>566.58</v>
+        <v>802.34</v>
       </c>
       <c r="E19" s="21" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>670.5609741210938</v>
+        <v>1007.163208007812</v>
       </c>
       <c r="G19" s="14">
         <f>(F19-D19)/D19</f>
         <v/>
       </c>
       <c r="H19" s="14" t="n">
-        <v>0.9387755102040817</v>
+        <v>0.6071428571428571</v>
       </c>
       <c r="I19" s="16">
         <f>IF(G19&gt;=0.25, "HIGH CONVICTION CATALYST", IF(G19&gt;=0.10, "MONITORING CATALYST", "SECONDARY"))</f>
@@ -4178,21 +4178,21 @@
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="B20" s="12" t="inlineStr">
         <is>
-          <t>APPLE INC</t>
+          <t>CHEVRON CORP</t>
         </is>
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D20" s="13" t="n">
-        <v>333.63</v>
+        <v>211.69</v>
       </c>
       <c r="E20" s="21" t="inlineStr">
         <is>
@@ -4200,14 +4200,14 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>333.6066589355469</v>
+        <v>225.2142791748047</v>
       </c>
       <c r="G20" s="14">
         <f>(F20-D20)/D20</f>
         <v/>
       </c>
       <c r="H20" s="14" t="n">
-        <v>0.5892857142857143</v>
+        <v>0.8064516129032258</v>
       </c>
       <c r="I20" s="16">
         <f>IF(G20&gt;=0.25, "HIGH CONVICTION CATALYST", IF(G20&gt;=0.10, "MONITORING CATALYST", "SECONDARY"))</f>
@@ -4217,21 +4217,21 @@
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>CHEVRON CORP</t>
+          <t>AMAZON.COM INC</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D21" s="13" t="n">
-        <v>207.58</v>
+        <v>261.78</v>
       </c>
       <c r="E21" s="21" t="inlineStr">
         <is>
@@ -4239,14 +4239,14 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>224.0740814208984</v>
+        <v>332.6354675292969</v>
       </c>
       <c r="G21" s="14">
         <f>(F21-D21)/D21</f>
         <v/>
       </c>
       <c r="H21" s="14" t="n">
-        <v>0.8064516129032258</v>
+        <v>0.9506172839506173</v>
       </c>
       <c r="I21" s="16">
         <f>IF(G21&gt;=0.25, "HIGH CONVICTION CATALYST", IF(G21&gt;=0.10, "MONITORING CATALYST", "SECONDARY"))</f>
@@ -4256,21 +4256,21 @@
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>ABBV</t>
         </is>
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>AMAZON.COM INC</t>
+          <t>ABBVIE INC</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="D22" s="13" t="n">
-        <v>256.29</v>
+        <v>276.12</v>
       </c>
       <c r="E22" s="21" t="inlineStr">
         <is>
@@ -4278,14 +4278,14 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>332.6354675292969</v>
+        <v>283.1724243164062</v>
       </c>
       <c r="G22" s="14">
         <f>(F22-D22)/D22</f>
         <v/>
       </c>
       <c r="H22" s="14" t="n">
-        <v>0.9506172839506173</v>
+        <v>0.8181818181818182</v>
       </c>
       <c r="I22" s="16">
         <f>IF(G22&gt;=0.25, "HIGH CONVICTION CATALYST", IF(G22&gt;=0.10, "MONITORING CATALYST", "SECONDARY"))</f>
@@ -4295,36 +4295,36 @@
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>ABBV</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>ABBVIE INC</t>
+          <t>APPLE INC</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D23" s="13" t="n">
-        <v>266.69</v>
+        <v>337.0814</v>
       </c>
       <c r="E23" s="21" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-11-02</t>
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>281.4482727050781</v>
+        <v>333.6066589355469</v>
       </c>
       <c r="G23" s="14">
         <f>(F23-D23)/D23</f>
         <v/>
       </c>
       <c r="H23" s="14" t="n">
-        <v>0.8181818181818182</v>
+        <v>0.5892857142857143</v>
       </c>
       <c r="I23" s="16">
         <f>IF(G23&gt;=0.25, "HIGH CONVICTION CATALYST", IF(G23&gt;=0.10, "MONITORING CATALYST", "SECONDARY"))</f>
@@ -4348,11 +4348,11 @@
         </is>
       </c>
       <c r="D24" s="13" t="n">
-        <v>649.42</v>
+        <v>609.7431</v>
       </c>
       <c r="E24" s="21" t="inlineStr">
         <is>
-          <t>2026-11-04</t>
+          <t>2026-11-03</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
@@ -4373,21 +4373,21 @@
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>NVIDIA CORP</t>
+          <t>WALMART INC</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D25" s="13" t="n">
-        <v>239.24</v>
+        <v>111.145</v>
       </c>
       <c r="E25" s="21" t="inlineStr">
         <is>
@@ -4395,14 +4395,14 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>323.8887634277344</v>
+        <v>128.8444519042969</v>
       </c>
       <c r="G25" s="14">
         <f>(F25-D25)/D25</f>
         <v/>
       </c>
       <c r="H25" s="14" t="n">
-        <v>0.9634146341463414</v>
+        <v>0.8846153846153846</v>
       </c>
       <c r="I25" s="16">
         <f>IF(G25&gt;=0.25, "HIGH CONVICTION CATALYST", IF(G25&gt;=0.10, "MONITORING CATALYST", "SECONDARY"))</f>
@@ -4412,21 +4412,21 @@
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>WALMART INC</t>
+          <t>NVIDIA CORP</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D26" s="13" t="n">
-        <v>107.2</v>
+        <v>229.785</v>
       </c>
       <c r="E26" s="21" t="inlineStr">
         <is>
@@ -4434,14 +4434,14 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>128.2888946533203</v>
+        <v>324.6381530761719</v>
       </c>
       <c r="G26" s="14">
         <f>(F26-D26)/D26</f>
         <v/>
       </c>
       <c r="H26" s="14" t="n">
-        <v>0.8846153846153846</v>
+        <v>0.9634146341463414</v>
       </c>
       <c r="I26" s="16">
         <f>IF(G26&gt;=0.25, "HIGH CONVICTION CATALYST", IF(G26&gt;=0.10, "MONITORING CATALYST", "SECONDARY"))</f>
@@ -4465,7 +4465,7 @@
         </is>
       </c>
       <c r="D27" s="13" t="n">
-        <v>164.48</v>
+        <v>168.77</v>
       </c>
       <c r="E27" s="21" t="inlineStr">
         <is>
@@ -4473,7 +4473,7 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>172.4400024414062</v>
+        <v>172.6399993896484</v>
       </c>
       <c r="G27" s="14">
         <f>(F27-D27)/D27</f>
@@ -4504,7 +4504,7 @@
         </is>
       </c>
       <c r="D28" s="13" t="n">
-        <v>935.6799999999999</v>
+        <v>946.9</v>
       </c>
       <c r="E28" s="21" t="inlineStr">
         <is>
@@ -4512,7 +4512,7 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>1074.228515625</v>
+        <v>1077.085693359375</v>
       </c>
       <c r="G28" s="14">
         <f>(F28-D28)/D28</f>
@@ -4543,7 +4543,7 @@
         </is>
       </c>
       <c r="D29" s="13" t="n">
-        <v>375.81</v>
+        <v>362.57</v>
       </c>
       <c r="E29" s="21" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add news intelligence terminal, executive rough summaries, and watchlist change flags
</commit_message>
<xml_diff>
--- a/bloomberg_live_remote_dashboard.xlsx
+++ b/bloomberg_live_remote_dashboard.xlsx
@@ -598,7 +598,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Strategy Playbook &amp; Mathematical Risk Framework | Synced: 2026-10-09 14:47:38</t>
+          <t>Strategy Playbook &amp; Mathematical Risk Framework | Synced: 2026-10-09 15:43:58</t>
         </is>
       </c>
     </row>
@@ -868,7 +868,7 @@
     <col width="15" customWidth="1" min="17" max="17"/>
     <col width="21" customWidth="1" min="18" max="18"/>
     <col width="21" customWidth="1" min="19" max="19"/>
-    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="21" customWidth="1" min="20" max="20"/>
     <col width="13" customWidth="1" min="21" max="21"/>
     <col width="16" customWidth="1" min="22" max="22"/>
   </cols>
@@ -1017,13 +1017,13 @@
         </is>
       </c>
       <c r="D5" s="13" t="n">
-        <v>362.57</v>
+        <v>361.54</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>0.006747376</v>
+        <v>0.003887377</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>0.02092133</v>
+        <v>0.01802106</v>
       </c>
       <c r="G5" s="13" t="n">
         <v>529.7020874023438</v>
@@ -1069,13 +1069,13 @@
         <v>44.24543410014627</v>
       </c>
       <c r="S5" s="19" t="n">
-        <v>43.49197309083039</v>
+        <v>43.3684199058238</v>
       </c>
       <c r="T5" s="20" t="n">
-        <v>1730774980153.05</v>
+        <v>1725858141392.1</v>
       </c>
       <c r="U5" s="17" t="n">
-        <v>12447287</v>
+        <v>16423255</v>
       </c>
       <c r="V5" s="21" t="inlineStr">
         <is>
@@ -1100,13 +1100,13 @@
         </is>
       </c>
       <c r="D6" s="13" t="n">
-        <v>229.785</v>
+        <v>229.28</v>
       </c>
       <c r="E6" s="14" t="n">
-        <v>-0.003015446</v>
+        <v>-0.005206526</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>-0.01780295</v>
+        <v>-0.01996153</v>
       </c>
       <c r="G6" s="13" t="n">
         <v>324.6381530761719</v>
@@ -1152,13 +1152,13 @@
         <v>117.210701426553</v>
       </c>
       <c r="S6" s="19" t="n">
-        <v>33.04229915529706</v>
+        <v>32.96968117698324</v>
       </c>
       <c r="T6" s="20" t="n">
-        <v>5537818500000</v>
+        <v>5525648000000</v>
       </c>
       <c r="U6" s="17" t="n">
-        <v>64209802</v>
+        <v>84205379</v>
       </c>
       <c r="V6" s="21" t="inlineStr">
         <is>
@@ -1183,13 +1183,13 @@
         </is>
       </c>
       <c r="D7" s="13" t="n">
-        <v>307.865</v>
+        <v>308.2</v>
       </c>
       <c r="E7" s="14" t="n">
-        <v>0.007345722999999999</v>
+        <v>0.008441855999999999</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>-0.005475514</v>
+        <v>-0.004393332</v>
       </c>
       <c r="G7" s="13" t="n">
         <v>393</v>
@@ -1235,13 +1235,13 @@
         <v>48.79401767505099</v>
       </c>
       <c r="S7" s="19" t="n">
-        <v>42.63271516035753</v>
+        <v>42.67910853662888</v>
       </c>
       <c r="T7" s="20" t="n">
-        <v>319429183064.745</v>
+        <v>319776766506.6</v>
       </c>
       <c r="U7" s="17" t="n">
-        <v>1844198</v>
+        <v>2946918</v>
       </c>
       <c r="V7" s="21" t="inlineStr">
         <is>
@@ -1266,13 +1266,13 @@
         </is>
       </c>
       <c r="D8" s="13" t="n">
-        <v>261.78</v>
+        <v>262.43</v>
       </c>
       <c r="E8" s="14" t="n">
-        <v>0.03038652</v>
+        <v>0.03294497</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>0.04079198</v>
+        <v>0.04337627</v>
       </c>
       <c r="G8" s="13" t="n">
         <v>332.6354675292969</v>
@@ -1318,13 +1318,13 @@
         <v>30.55833836875067</v>
       </c>
       <c r="S8" s="19" t="n">
-        <v>36.36815256498377</v>
+        <v>36.45845387640514</v>
       </c>
       <c r="T8" s="20" t="n">
-        <v>2823641166878.16</v>
+        <v>2830652270699.959</v>
       </c>
       <c r="U8" s="17" t="n">
-        <v>24552192</v>
+        <v>33436615</v>
       </c>
       <c r="V8" s="21" t="inlineStr">
         <is>
@@ -1349,13 +1349,13 @@
         </is>
       </c>
       <c r="D9" s="13" t="n">
-        <v>381.71</v>
+        <v>379.3</v>
       </c>
       <c r="E9" s="14" t="n">
-        <v>0.0290066</v>
+        <v>0.02250977</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>0.02637806</v>
+        <v>0.01989782</v>
       </c>
       <c r="G9" s="13" t="n">
         <v>480.0740661621094</v>
@@ -1401,13 +1401,13 @@
         <v>14.62124231898163</v>
       </c>
       <c r="S9" s="19" t="n">
-        <v>21.43376701117273</v>
+        <v>21.29844056401107</v>
       </c>
       <c r="T9" s="20" t="n">
-        <v>342620929048.37</v>
+        <v>340457725467.1</v>
       </c>
       <c r="U9" s="17" t="n">
-        <v>5250799</v>
+        <v>7439236</v>
       </c>
       <c r="V9" s="21" t="inlineStr">
         <is>
@@ -1432,13 +1432,13 @@
         </is>
       </c>
       <c r="D10" s="13" t="n">
-        <v>802.34</v>
+        <v>800.47</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>0.007736944</v>
+        <v>0.005388229</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>-0.05095692</v>
+        <v>-0.05316884</v>
       </c>
       <c r="G10" s="13" t="n">
         <v>1007.163208007812</v>
@@ -1484,13 +1484,13 @@
         <v>56.98969939037208</v>
       </c>
       <c r="S10" s="19" t="n">
-        <v>34.12093026696047</v>
+        <v>34.04140281795672</v>
       </c>
       <c r="T10" s="20" t="n">
-        <v>368815550440.26</v>
+        <v>367955958397.83</v>
       </c>
       <c r="U10" s="17" t="n">
-        <v>1027301</v>
+        <v>1526727</v>
       </c>
       <c r="V10" s="21" t="inlineStr">
         <is>
@@ -1501,30 +1501,30 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>LMT</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>LOCKHEED MARTIN CORP</t>
+          <t>GOLDMAN SACHS GROUP INC</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D11" s="13" t="n">
-        <v>509.29</v>
+        <v>895.3200000000001</v>
       </c>
       <c r="E11" s="14" t="n">
-        <v>0.002756502</v>
+        <v>0.01442346</v>
       </c>
       <c r="F11" s="14" t="n">
-        <v>0.007676936</v>
+        <v>-0.008021627</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>634.0416870117188</v>
+        <v>1116</v>
       </c>
       <c r="H11" s="14">
         <f>(G11-D11)/D11</f>
@@ -1551,10 +1551,10 @@
         <v/>
       </c>
       <c r="N11" s="17" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="O11" s="17" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="P11" s="17" t="n">
         <v>1</v>
@@ -1564,50 +1564,50 @@
         <v/>
       </c>
       <c r="R11" s="18" t="n">
-        <v>89.16465749539071</v>
+        <v>18.3355666637702</v>
       </c>
       <c r="S11" s="19" t="n">
-        <v>23.50835059235798</v>
+        <v>13.6932330607338</v>
       </c>
       <c r="T11" s="20" t="n">
-        <v>117539422595.37</v>
+        <v>271034247339</v>
       </c>
       <c r="U11" s="17" t="n">
-        <v>519730</v>
+        <v>1856475</v>
       </c>
       <c r="V11" s="21" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>LMT</t>
         </is>
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>GOLDMAN SACHS GROUP INC</t>
+          <t>LOCKHEED MARTIN CORP</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D12" s="13" t="n">
-        <v>897.14</v>
+        <v>509.59</v>
       </c>
       <c r="E12" s="14" t="n">
-        <v>0.01648557</v>
+        <v>0.003347181</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>-0.006005141</v>
+        <v>0.008270513</v>
       </c>
       <c r="G12" s="13" t="n">
-        <v>1116</v>
+        <v>634.0416870117188</v>
       </c>
       <c r="H12" s="14">
         <f>(G12-D12)/D12</f>
@@ -1634,10 +1634,10 @@
         <v/>
       </c>
       <c r="N12" s="17" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="O12" s="17" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="P12" s="17" t="n">
         <v>1</v>
@@ -1647,20 +1647,20 @@
         <v/>
       </c>
       <c r="R12" s="18" t="n">
-        <v>18.3355666637702</v>
+        <v>89.16465749539071</v>
       </c>
       <c r="S12" s="19" t="n">
-        <v>13.72106867733892</v>
+        <v>23.52219774838346</v>
       </c>
       <c r="T12" s="20" t="n">
-        <v>271585203790.5</v>
+        <v>117608659821.27</v>
       </c>
       <c r="U12" s="17" t="n">
-        <v>1280873</v>
+        <v>801202</v>
       </c>
       <c r="V12" s="21" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -1681,13 +1681,13 @@
         </is>
       </c>
       <c r="D13" s="13" t="n">
-        <v>185.75</v>
+        <v>185.97</v>
       </c>
       <c r="E13" s="14" t="n">
-        <v>0.007758247</v>
+        <v>0.008951822999999999</v>
       </c>
       <c r="F13" s="14" t="n">
-        <v>0.005793806</v>
+        <v>0.006985055</v>
       </c>
       <c r="G13" s="13" t="n">
         <v>229.625</v>
@@ -1733,13 +1733,13 @@
         <v>12.01786060959037</v>
       </c>
       <c r="S13" s="19" t="n">
-        <v>26.84646208434053</v>
+        <v>26.87825887804236</v>
       </c>
       <c r="T13" s="20" t="n">
-        <v>250346075248</v>
+        <v>250642582039.68</v>
       </c>
       <c r="U13" s="17" t="n">
-        <v>2282384</v>
+        <v>3344658</v>
       </c>
       <c r="V13" s="21" t="inlineStr">
         <is>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D14" s="13" t="n">
-        <v>351.23</v>
+        <v>351.66</v>
       </c>
       <c r="E14" s="14" t="n">
-        <v>0.008441241</v>
+        <v>0.009675844999999999</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>0.02250364</v>
+        <v>0.02375546</v>
       </c>
       <c r="G14" s="13" t="n">
         <v>429.2468566894531</v>
@@ -1816,13 +1816,13 @@
         <v>49.54854659098636</v>
       </c>
       <c r="S14" s="19" t="n">
-        <v>33.95925807549528</v>
+        <v>34.00083263288126</v>
       </c>
       <c r="T14" s="20" t="n">
-        <v>4274231867500</v>
+        <v>4278212700000</v>
       </c>
       <c r="U14" s="17" t="n">
-        <v>11846311</v>
+        <v>17201442</v>
       </c>
       <c r="V14" s="21" t="inlineStr">
         <is>
@@ -1847,13 +1847,13 @@
         </is>
       </c>
       <c r="D15" s="13" t="n">
-        <v>111.145</v>
+        <v>111.35</v>
       </c>
       <c r="E15" s="14" t="n">
-        <v>0.005291245</v>
+        <v>0.007145441</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>0.06603683</v>
+        <v>0.06800307</v>
       </c>
       <c r="G15" s="13" t="n">
         <v>128.8444519042969</v>
@@ -1899,13 +1899,13 @@
         <v>23.4417142735787</v>
       </c>
       <c r="S15" s="19" t="n">
-        <v>39.29485857388293</v>
+        <v>39.36733613204554</v>
       </c>
       <c r="T15" s="20" t="n">
-        <v>881796225955.9449</v>
+        <v>883422643935.3499</v>
       </c>
       <c r="U15" s="17" t="n">
-        <v>7916610</v>
+        <v>11817135</v>
       </c>
       <c r="V15" s="21" t="inlineStr">
         <is>
@@ -1930,13 +1930,13 @@
         </is>
       </c>
       <c r="D16" s="13" t="n">
-        <v>1175.95</v>
+        <v>1179.27</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>0.005429207</v>
+        <v>0.008267784</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>0.02896268</v>
+        <v>0.0318677</v>
       </c>
       <c r="G16" s="13" t="n">
         <v>1347.217529296875</v>
@@ -1982,13 +1982,13 @@
         <v>102.4296334361739</v>
       </c>
       <c r="S16" s="19" t="n">
-        <v>33.02816049054621</v>
+        <v>33.12140914496705</v>
       </c>
       <c r="T16" s="20" t="n">
-        <v>1106988840586.75</v>
+        <v>1110114146042.55</v>
       </c>
       <c r="U16" s="17" t="n">
-        <v>924530</v>
+        <v>1383717</v>
       </c>
       <c r="V16" s="21" t="inlineStr">
         <is>
@@ -2013,13 +2013,13 @@
         </is>
       </c>
       <c r="D17" s="13" t="n">
-        <v>588.925</v>
+        <v>589.14</v>
       </c>
       <c r="E17" s="14" t="n">
-        <v>0.0261984</v>
+        <v>0.02657304</v>
       </c>
       <c r="F17" s="14" t="n">
-        <v>0.06639083</v>
+        <v>0.06678014</v>
       </c>
       <c r="G17" s="13" t="n">
         <v>670.6666870117188</v>
@@ -2065,13 +2065,13 @@
         <v>241.4884135472371</v>
       </c>
       <c r="S17" s="19" t="n">
-        <v>31.06309595958312</v>
+        <v>31.07443764143354</v>
       </c>
       <c r="T17" s="20" t="n">
-        <v>516017133286.5</v>
+        <v>516205516669.2</v>
       </c>
       <c r="U17" s="17" t="n">
-        <v>1543688</v>
+        <v>2423215</v>
       </c>
       <c r="V17" s="21" t="inlineStr">
         <is>
@@ -2096,13 +2096,13 @@
         </is>
       </c>
       <c r="D18" s="13" t="n">
-        <v>946.9</v>
+        <v>946.92</v>
       </c>
       <c r="E18" s="14" t="n">
-        <v>-0.00107604</v>
+        <v>-0.001054941</v>
       </c>
       <c r="F18" s="14" t="n">
-        <v>0.02851246</v>
+        <v>0.02853419</v>
       </c>
       <c r="G18" s="13" t="n">
         <v>1077.085693359375</v>
@@ -2148,13 +2148,13 @@
         <v>28.4021118413964</v>
       </c>
       <c r="S18" s="19" t="n">
-        <v>45.61394735710621</v>
+        <v>45.61490879523767</v>
       </c>
       <c r="T18" s="20" t="n">
-        <v>419599180568.1</v>
+        <v>419608043155.08</v>
       </c>
       <c r="U18" s="17" t="n">
-        <v>924736</v>
+        <v>1485525</v>
       </c>
       <c r="V18" s="21" t="inlineStr">
         <is>
@@ -2179,13 +2179,13 @@
         </is>
       </c>
       <c r="D19" s="13" t="n">
-        <v>333.34</v>
+        <v>332.99</v>
       </c>
       <c r="E19" s="14" t="n">
-        <v>0.005793253000000001</v>
+        <v>0.004737191</v>
       </c>
       <c r="F19" s="14" t="n">
-        <v>0.00288826</v>
+        <v>0.001835249</v>
       </c>
       <c r="G19" s="13" t="n">
         <v>371.4003601074219</v>
@@ -2231,13 +2231,13 @@
         <v>18.4323841277336</v>
       </c>
       <c r="S19" s="19" t="n">
-        <v>14.17862491402675</v>
+        <v>14.16373739583545</v>
       </c>
       <c r="T19" s="20" t="n">
-        <v>886079786241.2998</v>
+        <v>885149421073.05</v>
       </c>
       <c r="U19" s="17" t="n">
-        <v>3168300</v>
+        <v>4917943</v>
       </c>
       <c r="V19" s="21" t="inlineStr">
         <is>
@@ -2262,13 +2262,13 @@
         </is>
       </c>
       <c r="D20" s="13" t="n">
-        <v>719.36</v>
+        <v>718.67</v>
       </c>
       <c r="E20" s="14" t="n">
-        <v>-0.002122377</v>
+        <v>-0.003079527</v>
       </c>
       <c r="F20" s="14" t="n">
-        <v>-0.01197671</v>
+        <v>-0.0129244</v>
       </c>
       <c r="G20" s="13" t="n">
         <v>795.2846069335938</v>
@@ -2314,13 +2314,13 @@
         <v>29.84849580640424</v>
       </c>
       <c r="S20" s="19" t="n">
-        <v>21.29844122656482</v>
+        <v>21.27801198843129</v>
       </c>
       <c r="T20" s="20" t="n">
-        <v>1832574078016</v>
+        <v>1830816298720.75</v>
       </c>
       <c r="U20" s="17" t="n">
-        <v>9992704</v>
+        <v>12554878</v>
       </c>
       <c r="V20" s="21" t="inlineStr">
         <is>
@@ -2345,13 +2345,13 @@
         </is>
       </c>
       <c r="D21" s="13" t="n">
-        <v>385.245</v>
+        <v>385.45</v>
       </c>
       <c r="E21" s="14" t="n">
-        <v>0.02704612</v>
+        <v>0.02759264</v>
       </c>
       <c r="F21" s="14" t="n">
-        <v>0.06816669</v>
+        <v>0.06873509999999999</v>
       </c>
       <c r="G21" s="13" t="n">
         <v>424.2857055664063</v>
@@ -2397,13 +2397,13 @@
         <v>62.35974440012697</v>
       </c>
       <c r="S21" s="19" t="n">
-        <v>32.354005126586</v>
+        <v>32.37122306337925</v>
       </c>
       <c r="T21" s="20" t="n">
-        <v>719295890683.2638</v>
+        <v>719678648817.9313</v>
       </c>
       <c r="U21" s="17" t="n">
-        <v>3837920</v>
+        <v>5815546</v>
       </c>
       <c r="V21" s="21" t="inlineStr">
         <is>
@@ -2414,30 +2414,30 @@
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>JNJ</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>JOHNSON &amp; JOHNSON</t>
+          <t>MICROSOFT CORP</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D22" s="13" t="n">
-        <v>260.28</v>
+        <v>535.0700000000001</v>
       </c>
       <c r="E22" s="14" t="n">
-        <v>0.01481597</v>
+        <v>0.02384187</v>
       </c>
       <c r="F22" s="14" t="n">
-        <v>0.01659962</v>
+        <v>0.03389176</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>284.2000122070312</v>
+        <v>582.3107299804688</v>
       </c>
       <c r="H22" s="14">
         <f>(G22-D22)/D22</f>
@@ -2464,10 +2464,10 @@
         <v/>
       </c>
       <c r="N22" s="17" t="n">
-        <v>20</v>
+        <v>70</v>
       </c>
       <c r="O22" s="17" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="P22" s="17" t="n">
         <v>0</v>
@@ -2477,50 +2477,50 @@
         <v/>
       </c>
       <c r="R22" s="18" t="n">
-        <v>25.74215021658794</v>
+        <v>34.03862745048138</v>
       </c>
       <c r="S22" s="19" t="n">
-        <v>28.08244105975901</v>
+        <v>32.24684176424994</v>
       </c>
       <c r="T22" s="20" t="n">
-        <v>627248406827.1599</v>
+        <v>3973186625869.37</v>
       </c>
       <c r="U22" s="17" t="n">
-        <v>3305448</v>
+        <v>17819581</v>
       </c>
       <c r="V22" s="21" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>JNJ</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>MICROSOFT CORP</t>
+          <t>JOHNSON &amp; JOHNSON</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="D23" s="13" t="n">
-        <v>535.4109999999999</v>
+        <v>261.44</v>
       </c>
       <c r="E23" s="14" t="n">
-        <v>0.02449436</v>
+        <v>0.01933874</v>
       </c>
       <c r="F23" s="14" t="n">
-        <v>0.03455065</v>
+        <v>0.02113034</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>582.3107299804688</v>
+        <v>284.2000122070312</v>
       </c>
       <c r="H23" s="14">
         <f>(G23-D23)/D23</f>
@@ -2547,10 +2547,10 @@
         <v/>
       </c>
       <c r="N23" s="17" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="O23" s="17" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="P23" s="17" t="n">
         <v>0</v>
@@ -2560,20 +2560,20 @@
         <v/>
       </c>
       <c r="R23" s="18" t="n">
-        <v>34.03862745048138</v>
+        <v>25.74215021658794</v>
       </c>
       <c r="S23" s="19" t="n">
-        <v>32.2673928755247</v>
+        <v>28.20759756284441</v>
       </c>
       <c r="T23" s="20" t="n">
-        <v>3975718736881.8</v>
+        <v>630043889199.6799</v>
       </c>
       <c r="U23" s="17" t="n">
-        <v>12457020</v>
+        <v>5459240</v>
       </c>
       <c r="V23" s="21" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -2594,13 +2594,13 @@
         </is>
       </c>
       <c r="D24" s="13" t="n">
-        <v>609.7431</v>
+        <v>608.1</v>
       </c>
       <c r="E24" s="14" t="n">
-        <v>-0.01762084</v>
+        <v>-0.02026809</v>
       </c>
       <c r="F24" s="14" t="n">
-        <v>-0.03812355</v>
+        <v>-0.04071556</v>
       </c>
       <c r="G24" s="13" t="n">
         <v>648.9697875976562</v>
@@ -2646,13 +2646,13 @@
         <v>10.14114698673644</v>
       </c>
       <c r="S24" s="19" t="n">
-        <v>169.2992508898463</v>
+        <v>168.8430255654999</v>
       </c>
       <c r="T24" s="20" t="n">
-        <v>995390392781.7102</v>
+        <v>992708073040.2</v>
       </c>
       <c r="U24" s="17" t="n">
-        <v>10939958</v>
+        <v>13623783</v>
       </c>
       <c r="V24" s="21" t="inlineStr">
         <is>
@@ -2677,13 +2677,13 @@
         </is>
       </c>
       <c r="D25" s="13" t="n">
-        <v>211.69</v>
+        <v>211.98</v>
       </c>
       <c r="E25" s="14" t="n">
-        <v>0.0006617821</v>
+        <v>0.002032616</v>
       </c>
       <c r="F25" s="14" t="n">
-        <v>0.02419082</v>
+        <v>0.02559388</v>
       </c>
       <c r="G25" s="13" t="n">
         <v>225.2142791748047</v>
@@ -2729,13 +2729,13 @@
         <v>12.24561403508772</v>
       </c>
       <c r="S25" s="19" t="n">
-        <v>20.6584937442801</v>
+        <v>20.68679373208475</v>
       </c>
       <c r="T25" s="20" t="n">
-        <v>418251020993.06</v>
+        <v>418823994662.52</v>
       </c>
       <c r="U25" s="17" t="n">
-        <v>3943646</v>
+        <v>6020412</v>
       </c>
       <c r="V25" s="21" t="inlineStr">
         <is>
@@ -2760,13 +2760,13 @@
         </is>
       </c>
       <c r="D26" s="13" t="n">
-        <v>383.97</v>
+        <v>382.7</v>
       </c>
       <c r="E26" s="14" t="n">
-        <v>0.02392</v>
+        <v>0.02053333</v>
       </c>
       <c r="F26" s="14" t="n">
-        <v>0.03610459</v>
+        <v>0.03267762</v>
       </c>
       <c r="G26" s="13" t="n">
         <v>397.1675109863281</v>
@@ -2812,13 +2812,13 @@
         <v>4.636600638354896</v>
       </c>
       <c r="S26" s="19" t="n">
-        <v>384.1175023416023</v>
+        <v>382.8470254648097</v>
       </c>
       <c r="T26" s="20" t="n">
-        <v>1516507712874.18</v>
+        <v>1511491787683.8</v>
       </c>
       <c r="U26" s="17" t="n">
-        <v>33777365</v>
+        <v>38782597</v>
       </c>
       <c r="V26" s="21" t="inlineStr">
         <is>
@@ -2843,13 +2843,13 @@
         </is>
       </c>
       <c r="D27" s="13" t="n">
-        <v>276.12</v>
+        <v>276.47</v>
       </c>
       <c r="E27" s="14" t="n">
-        <v>0.01358197</v>
+        <v>0.01486675</v>
       </c>
       <c r="F27" s="14" t="n">
-        <v>0.05060498</v>
+        <v>0.05193669</v>
       </c>
       <c r="G27" s="13" t="n">
         <v>283.1724243164062</v>
@@ -2895,13 +2895,13 @@
         <v>0</v>
       </c>
       <c r="S27" s="19" t="n">
-        <v>27.19939556081934</v>
+        <v>27.23387315978562</v>
       </c>
       <c r="T27" s="20" t="n">
-        <v>487936424734.2</v>
+        <v>488554915783.95</v>
       </c>
       <c r="U27" s="17" t="n">
-        <v>2057977</v>
+        <v>4262958</v>
       </c>
       <c r="V27" s="21" t="inlineStr">
         <is>
@@ -2926,13 +2926,13 @@
         </is>
       </c>
       <c r="D28" s="13" t="n">
-        <v>168.77</v>
+        <v>168.94</v>
       </c>
       <c r="E28" s="14" t="n">
-        <v>0.001602374</v>
+        <v>0.002611276</v>
       </c>
       <c r="F28" s="14" t="n">
-        <v>0.02902262</v>
+        <v>0.03005914</v>
       </c>
       <c r="G28" s="13" t="n">
         <v>172.6399993896484</v>
@@ -2978,13 +2978,13 @@
         <v>12.5512239138806</v>
       </c>
       <c r="S28" s="19" t="n">
-        <v>20.36142699522687</v>
+        <v>20.38193659538493</v>
       </c>
       <c r="T28" s="20" t="n">
-        <v>699459764861.2001</v>
+        <v>700164322306.4</v>
       </c>
       <c r="U28" s="17" t="n">
-        <v>5493118</v>
+        <v>8078028</v>
       </c>
       <c r="V28" s="21" t="inlineStr">
         <is>
@@ -3009,13 +3009,13 @@
         </is>
       </c>
       <c r="D29" s="13" t="n">
-        <v>337.0814</v>
+        <v>336.64</v>
       </c>
       <c r="E29" s="14" t="n">
-        <v>-0.009807297</v>
+        <v>-0.01110393</v>
       </c>
       <c r="F29" s="14" t="n">
-        <v>0.01016333</v>
+        <v>0.008840541</v>
       </c>
       <c r="G29" s="13" t="n">
         <v>333.6066589355469</v>
@@ -3061,13 +3061,13 @@
         <v>148.7510816267667</v>
       </c>
       <c r="S29" s="19" t="n">
-        <v>38.65612275009856</v>
+        <v>38.60550626702265</v>
       </c>
       <c r="T29" s="20" t="n">
-        <v>4919426626251.999</v>
+        <v>4912984755200</v>
       </c>
       <c r="U29" s="17" t="n">
-        <v>29097798</v>
+        <v>37765791</v>
       </c>
       <c r="V29" s="21" t="inlineStr">
         <is>
@@ -3607,7 +3607,7 @@
         </is>
       </c>
       <c r="D5" s="13" t="n">
-        <v>333.34</v>
+        <v>332.99</v>
       </c>
       <c r="E5" s="21" t="inlineStr">
         <is>
@@ -3646,7 +3646,7 @@
         </is>
       </c>
       <c r="D6" s="13" t="n">
-        <v>260.28</v>
+        <v>261.44</v>
       </c>
       <c r="E6" s="21" t="inlineStr">
         <is>
@@ -3685,7 +3685,7 @@
         </is>
       </c>
       <c r="D7" s="13" t="n">
-        <v>897.14</v>
+        <v>895.3200000000001</v>
       </c>
       <c r="E7" s="21" t="inlineStr">
         <is>
@@ -3724,7 +3724,7 @@
         </is>
       </c>
       <c r="D8" s="13" t="n">
-        <v>381.71</v>
+        <v>379.3</v>
       </c>
       <c r="E8" s="21" t="inlineStr">
         <is>
@@ -3763,7 +3763,7 @@
         </is>
       </c>
       <c r="D9" s="13" t="n">
-        <v>185.75</v>
+        <v>185.97</v>
       </c>
       <c r="E9" s="21" t="inlineStr">
         <is>
@@ -3802,7 +3802,7 @@
         </is>
       </c>
       <c r="D10" s="13" t="n">
-        <v>307.865</v>
+        <v>308.2</v>
       </c>
       <c r="E10" s="21" t="inlineStr">
         <is>
@@ -3841,7 +3841,7 @@
         </is>
       </c>
       <c r="D11" s="13" t="n">
-        <v>383.97</v>
+        <v>382.7</v>
       </c>
       <c r="E11" s="21" t="inlineStr">
         <is>
@@ -3880,7 +3880,7 @@
         </is>
       </c>
       <c r="D12" s="13" t="n">
-        <v>509.29</v>
+        <v>509.59</v>
       </c>
       <c r="E12" s="21" t="inlineStr">
         <is>
@@ -3919,7 +3919,7 @@
         </is>
       </c>
       <c r="D13" s="13" t="n">
-        <v>385.245</v>
+        <v>385.45</v>
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
@@ -3958,7 +3958,7 @@
         </is>
       </c>
       <c r="D14" s="13" t="n">
-        <v>351.23</v>
+        <v>351.66</v>
       </c>
       <c r="E14" s="21" t="inlineStr">
         <is>
@@ -3997,7 +3997,7 @@
         </is>
       </c>
       <c r="D15" s="13" t="n">
-        <v>535.4109999999999</v>
+        <v>535.0700000000001</v>
       </c>
       <c r="E15" s="21" t="inlineStr">
         <is>
@@ -4036,7 +4036,7 @@
         </is>
       </c>
       <c r="D16" s="13" t="n">
-        <v>719.36</v>
+        <v>718.67</v>
       </c>
       <c r="E16" s="21" t="inlineStr">
         <is>
@@ -4075,7 +4075,7 @@
         </is>
       </c>
       <c r="D17" s="13" t="n">
-        <v>1175.95</v>
+        <v>1179.27</v>
       </c>
       <c r="E17" s="21" t="inlineStr">
         <is>
@@ -4114,7 +4114,7 @@
         </is>
       </c>
       <c r="D18" s="13" t="n">
-        <v>588.925</v>
+        <v>589.14</v>
       </c>
       <c r="E18" s="21" t="inlineStr">
         <is>
@@ -4153,7 +4153,7 @@
         </is>
       </c>
       <c r="D19" s="13" t="n">
-        <v>802.34</v>
+        <v>800.47</v>
       </c>
       <c r="E19" s="21" t="inlineStr">
         <is>
@@ -4192,7 +4192,7 @@
         </is>
       </c>
       <c r="D20" s="13" t="n">
-        <v>211.69</v>
+        <v>211.98</v>
       </c>
       <c r="E20" s="21" t="inlineStr">
         <is>
@@ -4231,7 +4231,7 @@
         </is>
       </c>
       <c r="D21" s="13" t="n">
-        <v>261.78</v>
+        <v>262.43</v>
       </c>
       <c r="E21" s="21" t="inlineStr">
         <is>
@@ -4270,7 +4270,7 @@
         </is>
       </c>
       <c r="D22" s="13" t="n">
-        <v>276.12</v>
+        <v>276.47</v>
       </c>
       <c r="E22" s="21" t="inlineStr">
         <is>
@@ -4309,7 +4309,7 @@
         </is>
       </c>
       <c r="D23" s="13" t="n">
-        <v>337.0814</v>
+        <v>336.64</v>
       </c>
       <c r="E23" s="21" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="D24" s="13" t="n">
-        <v>609.7431</v>
+        <v>608.1</v>
       </c>
       <c r="E24" s="21" t="inlineStr">
         <is>
@@ -4387,7 +4387,7 @@
         </is>
       </c>
       <c r="D25" s="13" t="n">
-        <v>111.145</v>
+        <v>111.35</v>
       </c>
       <c r="E25" s="21" t="inlineStr">
         <is>
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="D26" s="13" t="n">
-        <v>229.785</v>
+        <v>229.28</v>
       </c>
       <c r="E26" s="21" t="inlineStr">
         <is>
@@ -4465,7 +4465,7 @@
         </is>
       </c>
       <c r="D27" s="13" t="n">
-        <v>168.77</v>
+        <v>168.94</v>
       </c>
       <c r="E27" s="21" t="inlineStr">
         <is>
@@ -4504,7 +4504,7 @@
         </is>
       </c>
       <c r="D28" s="13" t="n">
-        <v>946.9</v>
+        <v>946.92</v>
       </c>
       <c r="E28" s="21" t="inlineStr">
         <is>
@@ -4543,7 +4543,7 @@
         </is>
       </c>
       <c r="D29" s="13" t="n">
-        <v>362.57</v>
+        <v>361.54</v>
       </c>
       <c r="E29" s="21" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update terminal with 3-view navigation: read-only Current Holdings, empty-by-default Wishlist with 1-click add/remove, and 25-stock Screener Universe
</commit_message>
<xml_diff>
--- a/bloomberg_live_remote_dashboard.xlsx
+++ b/bloomberg_live_remote_dashboard.xlsx
@@ -598,7 +598,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Strategy Playbook &amp; Mathematical Risk Framework | Synced: 2026-10-09 15:43:58</t>
+          <t>Strategy Playbook &amp; Mathematical Risk Framework | Synced: 2026-10-09 15:46:02</t>
         </is>
       </c>
     </row>
@@ -1075,7 +1075,7 @@
         <v>1725858141392.1</v>
       </c>
       <c r="U5" s="17" t="n">
-        <v>16423255</v>
+        <v>16434596</v>
       </c>
       <c r="V5" s="21" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
         <v>5525648000000</v>
       </c>
       <c r="U6" s="17" t="n">
-        <v>84205379</v>
+        <v>84208320</v>
       </c>
       <c r="V6" s="21" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
         <v>319776766506.6</v>
       </c>
       <c r="U7" s="17" t="n">
-        <v>2946918</v>
+        <v>2947018</v>
       </c>
       <c r="V7" s="21" t="inlineStr">
         <is>
@@ -1324,7 +1324,7 @@
         <v>2830652270699.959</v>
       </c>
       <c r="U8" s="17" t="n">
-        <v>33436615</v>
+        <v>33438259</v>
       </c>
       <c r="V8" s="21" t="inlineStr">
         <is>
@@ -1407,7 +1407,7 @@
         <v>340457725467.1</v>
       </c>
       <c r="U9" s="17" t="n">
-        <v>7439236</v>
+        <v>7439250</v>
       </c>
       <c r="V9" s="21" t="inlineStr">
         <is>
@@ -1490,7 +1490,7 @@
         <v>367955958397.83</v>
       </c>
       <c r="U10" s="17" t="n">
-        <v>1526727</v>
+        <v>1526762</v>
       </c>
       <c r="V10" s="21" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
         <v>271034247339</v>
       </c>
       <c r="U11" s="17" t="n">
-        <v>1856475</v>
+        <v>1856539</v>
       </c>
       <c r="V11" s="21" t="inlineStr">
         <is>
@@ -1656,7 +1656,7 @@
         <v>117608659821.27</v>
       </c>
       <c r="U12" s="17" t="n">
-        <v>801202</v>
+        <v>801203</v>
       </c>
       <c r="V12" s="21" t="inlineStr">
         <is>
@@ -1739,7 +1739,7 @@
         <v>250642582039.68</v>
       </c>
       <c r="U13" s="17" t="n">
-        <v>3344658</v>
+        <v>3344676</v>
       </c>
       <c r="V13" s="21" t="inlineStr">
         <is>
@@ -1822,7 +1822,7 @@
         <v>4278212700000</v>
       </c>
       <c r="U14" s="17" t="n">
-        <v>17201442</v>
+        <v>17202095</v>
       </c>
       <c r="V14" s="21" t="inlineStr">
         <is>
@@ -1905,7 +1905,7 @@
         <v>883422643935.3499</v>
       </c>
       <c r="U15" s="17" t="n">
-        <v>11817135</v>
+        <v>11817164</v>
       </c>
       <c r="V15" s="21" t="inlineStr">
         <is>
@@ -1988,7 +1988,7 @@
         <v>1110114146042.55</v>
       </c>
       <c r="U16" s="17" t="n">
-        <v>1383717</v>
+        <v>1383742</v>
       </c>
       <c r="V16" s="21" t="inlineStr">
         <is>
@@ -2154,7 +2154,7 @@
         <v>419608043155.08</v>
       </c>
       <c r="U18" s="17" t="n">
-        <v>1485525</v>
+        <v>1490520</v>
       </c>
       <c r="V18" s="21" t="inlineStr">
         <is>
@@ -2237,7 +2237,7 @@
         <v>885149421073.05</v>
       </c>
       <c r="U19" s="17" t="n">
-        <v>4917943</v>
+        <v>4927391</v>
       </c>
       <c r="V19" s="21" t="inlineStr">
         <is>
@@ -2320,7 +2320,7 @@
         <v>1830816298720.75</v>
       </c>
       <c r="U20" s="17" t="n">
-        <v>12554878</v>
+        <v>12558684</v>
       </c>
       <c r="V20" s="21" t="inlineStr">
         <is>
@@ -2403,7 +2403,7 @@
         <v>719678648817.9313</v>
       </c>
       <c r="U21" s="17" t="n">
-        <v>5815546</v>
+        <v>5815548</v>
       </c>
       <c r="V21" s="21" t="inlineStr">
         <is>
@@ -2486,7 +2486,7 @@
         <v>3973186625869.37</v>
       </c>
       <c r="U22" s="17" t="n">
-        <v>17819581</v>
+        <v>17848535</v>
       </c>
       <c r="V22" s="21" t="inlineStr">
         <is>
@@ -2569,7 +2569,7 @@
         <v>630043889199.6799</v>
       </c>
       <c r="U23" s="17" t="n">
-        <v>5459240</v>
+        <v>5459241</v>
       </c>
       <c r="V23" s="21" t="inlineStr">
         <is>
@@ -2652,7 +2652,7 @@
         <v>992708073040.2</v>
       </c>
       <c r="U24" s="17" t="n">
-        <v>13623783</v>
+        <v>13624809</v>
       </c>
       <c r="V24" s="21" t="inlineStr">
         <is>
@@ -2735,7 +2735,7 @@
         <v>418823994662.52</v>
       </c>
       <c r="U25" s="17" t="n">
-        <v>6020412</v>
+        <v>6020845</v>
       </c>
       <c r="V25" s="21" t="inlineStr">
         <is>
@@ -2818,7 +2818,7 @@
         <v>1511491787683.8</v>
       </c>
       <c r="U26" s="17" t="n">
-        <v>38782597</v>
+        <v>38784295</v>
       </c>
       <c r="V26" s="21" t="inlineStr">
         <is>
@@ -2984,7 +2984,7 @@
         <v>700164322306.4</v>
       </c>
       <c r="U28" s="17" t="n">
-        <v>8078028</v>
+        <v>8078244</v>
       </c>
       <c r="V28" s="21" t="inlineStr">
         <is>
@@ -3067,7 +3067,7 @@
         <v>4912984755200</v>
       </c>
       <c r="U29" s="17" t="n">
-        <v>37765791</v>
+        <v>37770117</v>
       </c>
       <c r="V29" s="21" t="inlineStr">
         <is>

</xml_diff>